<commit_message>
Update data files and delete one image
</commit_message>
<xml_diff>
--- a/data/us_data_centers_FMV.xlsx
+++ b/data/us_data_centers_FMV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/richardevans/Docs/Economics/OSE/States/ME-DataCtrCostRev/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75EE7934-7E32-F44B-BBD9-F52B0EAAC1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D98E6A-F830-8349-B6E9-8BC84210C665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="56680" windowHeight="24280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="221">
   <si>
     <t>record_id</t>
   </si>
@@ -730,6 +730,30 @@
   </si>
   <si>
     <t>directory-style or secondary database source with useful figures but weaker provenance</t>
+  </si>
+  <si>
+    <t>FirstLight</t>
+  </si>
+  <si>
+    <t>Brunswick</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>$760,100 in tax abatement</t>
+  </si>
+  <si>
+    <t>Cumberland</t>
+  </si>
+  <si>
+    <t>Antin Infrastructure</t>
+  </si>
+  <si>
+    <t>See page 77 of https://www.brunswickme.gov/DocumentCenter/View/9923/2024-Personal-Property-Commitment-Book?bidId=</t>
+  </si>
+  <si>
+    <t>https://www.datacenter.fyi/public-record/cf045dc3</t>
   </si>
 </sst>
 </file>
@@ -834,7 +858,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -873,6 +897,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1175,7 +1211,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T22"/>
+  <dimension ref="A1:T23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2313,6 +2349,50 @@
         <v>175</v>
       </c>
     </row>
+    <row r="23" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="18">
+        <v>22</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="C23" t="s">
+        <v>218</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="H23" s="20">
+        <v>0.9</v>
+      </c>
+      <c r="I23">
+        <v>778600</v>
+      </c>
+      <c r="J23">
+        <v>18500</v>
+      </c>
+      <c r="K23" s="21">
+        <v>778600</v>
+      </c>
+      <c r="M23" t="s">
+        <v>216</v>
+      </c>
+      <c r="O23" t="s">
+        <v>220</v>
+      </c>
+      <c r="P23" t="s">
+        <v>219</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T22" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>